<commit_message>
Remove load and three body propagator, change propagator to proper n-body support driven by config file
</commit_message>
<xml_diff>
--- a/blend-vis/prelim_error_analysis.xlsx
+++ b/blend-vis/prelim_error_analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Desktop\MissionControl\blend-vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F2C245-649F-4ED7-8D47-57737FC46430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964AB7C4-F62D-485E-83C6-984D14841E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{232D07CE-A3A8-4A58-853A-52E372662423}"/>
   </bookViews>
@@ -267,10 +267,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$5:$B$7</c:f>
+              <c:f>Sheet1!$B$5:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>694397</c:v>
                 </c:pt>
@@ -280,15 +280,18 @@
                 <c:pt idx="2">
                   <c:v>69439681</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>694396801</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$P$5:$P$7</c:f>
+              <c:f>Sheet1!$P$5:$P$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>281017220.61019826</c:v>
                 </c:pt>
@@ -297,6 +300,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>989470.90552877588</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2922414.169849772</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -352,10 +358,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$5:$B$7</c:f>
+              <c:f>Sheet1!$B$5:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>694397</c:v>
                 </c:pt>
@@ -365,15 +371,18 @@
                 <c:pt idx="2">
                   <c:v>69439681</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>694396801</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$Q$5:$Q$7</c:f>
+              <c:f>Sheet1!$Q$5:$Q$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>263247451.22633642</c:v>
                 </c:pt>
@@ -382,6 +391,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>60907.532997690323</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>365130.23336050188</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -407,6 +419,7 @@
       <c:valAx>
         <c:axId val="1067058431"/>
         <c:scaling>
+          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -524,6 +537,7 @@
       <c:valAx>
         <c:axId val="1067058911"/>
         <c:scaling>
+          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -1283,14 +1297,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>138111</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>80961</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>180974</xdr:rowOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>123824</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1635,9 +1649,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D1DE5F3-31E3-4E3E-B740-DED204292403}">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
     <col min="12" max="14" width="12" bestFit="1" customWidth="1"/>
@@ -1908,6 +1923,67 @@
         <v>60907.532997690323</v>
       </c>
     </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>694396801</v>
+      </c>
+      <c r="C8">
+        <v>6039.5177818000002</v>
+      </c>
+      <c r="D8">
+        <v>30964314.060349599</v>
+      </c>
+      <c r="E8">
+        <v>-131933835.54998501</v>
+      </c>
+      <c r="F8">
+        <v>-57200538.005779602</v>
+      </c>
+      <c r="G8">
+        <v>385314.07221648598</v>
+      </c>
+      <c r="H8">
+        <v>6048.5749215713204</v>
+      </c>
+      <c r="I8">
+        <v>-31456.749819064498</v>
+      </c>
+      <c r="J8">
+        <f t="shared" ref="J8" si="8">ABS($B$1-D8)</f>
+        <v>2852659.9396504015</v>
+      </c>
+      <c r="K8">
+        <f t="shared" ref="K8" si="9">ABS($C$1-E8)</f>
+        <v>579634.54998500645</v>
+      </c>
+      <c r="L8">
+        <f t="shared" ref="L8" si="10">ABS($D$1-F8)</f>
+        <v>258572.30577959865</v>
+      </c>
+      <c r="M8">
+        <f t="shared" ref="M8" si="11">ABS($B$2-G8)</f>
+        <v>202198.77147720597</v>
+      </c>
+      <c r="N8">
+        <f t="shared" ref="N8" si="12">ABS($C$2-H8)</f>
+        <v>280175.86152614129</v>
+      </c>
+      <c r="O8">
+        <f t="shared" ref="O8" si="13">ABS($D$2-I8)</f>
+        <v>118056.04916770551</v>
+      </c>
+      <c r="P8">
+        <f t="shared" ref="P8" si="14">SQRT(POWER(J8,2)+POWER(K8,2)+POWER(L8,2))</f>
+        <v>2922414.169849772</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" ref="Q8" si="15">SQRT(POWER(M8,2)+POWER(N8,2)+POWER(O8,2))</f>
+        <v>365130.23336050188</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>